<commit_message>
Update planned outage input workbook
</commit_message>
<xml_diff>
--- a/Thesis Forecasting/outputs/outages_planning/Planned_Outages_Input.xlsx
+++ b/Thesis Forecasting/outputs/outages_planning/Planned_Outages_Input.xlsx
@@ -9,9 +9,7 @@
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$S$25</definedName>
-  </definedNames>
+  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -19,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -36,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -44,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -417,120 +427,99 @@
   </sheetPr>
   <dimension ref="A1:S25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="17" customWidth="1" min="4" max="4"/>
-    <col width="17" customWidth="1" min="5" max="5"/>
-    <col width="17" customWidth="1" min="6" max="6"/>
-    <col width="17" customWidth="1" min="7" max="7"/>
-    <col width="17" customWidth="1" min="8" max="8"/>
-    <col width="17" customWidth="1" min="9" max="9"/>
-    <col width="17" customWidth="1" min="10" max="10"/>
-    <col width="17" customWidth="1" min="11" max="11"/>
-    <col width="17" customWidth="1" min="12" max="12"/>
-    <col width="17" customWidth="1" min="13" max="13"/>
-    <col width="17" customWidth="1" min="14" max="14"/>
-    <col width="17" customWidth="1" min="15" max="15"/>
-    <col width="17" customWidth="1" min="16" max="16"/>
-    <col width="17" customWidth="1" min="17" max="17"/>
-    <col width="17" customWidth="1" min="18" max="18"/>
-    <col width="17" customWidth="1" min="19" max="19"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Hour</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>out_agus1_unit1</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>out_agus1_unit2</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>out_agus2_unit1</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>out_agus2_unit2</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>out_agus2_unit3</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>out_agus4_unit1</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>out_agus4_unit2</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>out_agus4_unit3</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>out_agus5_unit1</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>out_agus5_unit2</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>out_agus6_unit1</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>out_agus6_unit2</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>out_agus6_unit3</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>out_agus6_unit4</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>out_agus6_unit5</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>out_agus7_unit1</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>out_agus7_unit2</t>
         </is>
@@ -2049,7 +2038,6 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:S25"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>